<commit_message>
docs(ejecucion): saca el runner y las capturas de los reportes de Exportar CSV
Borra entrega-2/ejecucion/exp y entrega-2/evidencia, y quita de los reportes
los vínculos a capturas y scripts: lo observado queda en «Resultado obtenido».

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-2/04-ejecucion-exp.xlsx
+++ b/entrega-2/04-ejecucion-exp.xlsx
@@ -4947,7 +4947,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-009.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C40" s="10" t="n"/>
@@ -5686,7 +5686,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-010.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C40" s="10" t="n"/>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-011.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C39" s="10" t="n"/>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-012.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C39" s="10" t="n"/>
@@ -7882,7 +7882,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-013.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C41" s="10" t="n"/>
@@ -8640,7 +8640,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-014.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C41" s="10" t="n"/>
@@ -9381,7 +9381,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-015.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C40" s="10" t="n"/>
@@ -10120,7 +10120,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-016.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C40" s="10" t="n"/>
@@ -10769,7 +10769,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-017.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C34" s="10" t="n"/>
@@ -11418,7 +11418,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-018.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C34" s="10" t="n"/>
@@ -12009,7 +12009,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-001.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C31" s="10" t="n"/>
@@ -12761,7 +12761,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-019.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C40" s="10" t="n"/>
@@ -13418,7 +13418,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-020.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C34" s="10" t="n"/>
@@ -14050,7 +14050,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-021.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C33" s="10" t="n"/>
@@ -14697,7 +14697,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-022.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C34" s="10" t="n"/>
@@ -15376,7 +15376,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-023.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C36" s="10" t="n"/>
@@ -16055,7 +16055,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-024.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C36" s="10" t="n"/>
@@ -16792,7 +16792,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-025.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C40" s="10" t="n"/>
@@ -17527,7 +17527,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-026.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C40" s="10" t="n"/>
@@ -18285,7 +18285,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-027.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C41" s="10" t="n"/>
@@ -18945,7 +18945,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-028.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C35" s="10" t="n"/>
@@ -19544,7 +19544,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-002.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C32" s="10" t="n"/>
@@ -20202,7 +20202,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-029.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C35" s="10" t="n"/>
@@ -20881,7 +20881,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-030.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C36" s="10" t="n"/>
@@ -21562,7 +21562,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-031.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C36" s="10" t="n"/>
@@ -22241,7 +22241,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-032.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C36" s="10" t="n"/>
@@ -22920,7 +22920,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-033.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C36" s="10" t="n"/>
@@ -23599,7 +23599,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-034.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C36" s="10" t="n"/>
@@ -24278,7 +24278,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-035.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C36" s="10" t="n"/>
@@ -24958,7 +24958,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-036.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C36" s="10" t="n"/>
@@ -25628,7 +25628,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-037.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C35" s="10" t="n"/>
@@ -26296,7 +26296,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-038.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C35" s="10" t="n"/>
@@ -26935,7 +26935,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-003.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C34" s="10" t="n"/>
@@ -27636,7 +27636,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-039.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C36" s="10" t="n"/>
@@ -28349,7 +28349,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-040.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C38" s="10" t="n"/>
@@ -29070,7 +29070,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-041.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C38" s="10" t="n"/>
@@ -29791,7 +29791,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-042.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C38" s="10" t="n"/>
@@ -30474,7 +30474,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-043.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C36" s="10" t="n"/>
@@ -30906,7 +30906,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-044.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C21" s="10" t="n"/>
@@ -31571,7 +31571,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-045.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C36" s="10" t="n"/>
@@ -32262,7 +32262,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-046.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C36" s="10" t="n"/>
@@ -32967,7 +32967,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-047.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C38" s="10" t="n"/>
@@ -33643,7 +33643,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-048.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C35" s="10" t="n"/>
@@ -34225,7 +34225,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-004.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C31" s="10" t="n"/>
@@ -34860,7 +34860,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-049.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C34" s="10" t="n"/>
@@ -35499,7 +35499,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-050.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C34" s="10" t="n"/>
@@ -36168,7 +36168,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-051.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C35" s="10" t="n"/>
@@ -36800,7 +36800,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-052.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C33" s="10" t="n"/>
@@ -37430,7 +37430,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-053.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C33" s="10" t="n"/>
@@ -38071,7 +38071,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-054.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C34" s="10" t="n"/>
@@ -38699,7 +38699,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-055.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C33" s="10" t="n"/>
@@ -39331,7 +39331,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-056.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C33" s="10" t="n"/>
@@ -39978,7 +39978,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-057.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C34" s="10" t="n"/>
@@ -40676,7 +40676,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-058.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C37" s="10" t="n"/>
@@ -41264,7 +41264,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-005.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C31" s="10" t="n"/>
@@ -41939,7 +41939,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-059.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C36" s="10" t="n"/>
@@ -42573,7 +42573,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-060.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C33" s="10" t="n"/>
@@ -43203,7 +43203,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-061.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C33" s="10" t="n"/>
@@ -43834,7 +43834,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-062.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C33" s="10" t="n"/>
@@ -44566,7 +44566,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-063.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C39" s="10" t="n"/>
@@ -45364,7 +45364,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-064.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C43" s="10" t="n"/>
@@ -46066,7 +46066,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-065.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C37" s="10" t="n"/>
@@ -46738,7 +46738,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-066.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C35" s="10" t="n"/>
@@ -47436,7 +47436,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-067.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C37" s="10" t="n"/>
@@ -48256,7 +48256,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-068.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C44" s="10" t="n"/>
@@ -48890,7 +48890,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-006.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C33" s="10" t="n"/>
@@ -49533,7 +49533,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-069.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C35" s="10" t="n"/>
@@ -50178,7 +50178,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-070.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C35" s="10" t="n"/>
@@ -50952,7 +50952,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-071.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C41" s="10" t="n"/>
@@ -51764,7 +51764,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-072.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C43" s="10" t="n"/>
@@ -52422,7 +52422,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-073.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C34" s="10" t="n"/>
@@ -53062,7 +53062,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-074.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C34" s="10" t="n"/>
@@ -53718,7 +53718,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-075.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C35" s="10" t="n"/>
@@ -54489,7 +54489,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-007.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C42" s="10" t="n"/>
@@ -55279,7 +55279,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>evidencia/CP-EXP-008.jpg</t>
+          <t>Sin capturas: lo observado figura en "Resultado obtenido"</t>
         </is>
       </c>
       <c r="C43" s="10" t="n"/>

</xml_diff>